<commit_message>
Update Stage A and Stage B, add data and literature review docs
</commit_message>
<xml_diff>
--- a/EDA_Log.xlsx
+++ b/EDA_Log.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Firm</t>
   </si>
@@ -104,6 +104,21 @@
   </si>
   <si>
     <t>Appendix cell share 29%; pdfplumber detects gridlined tables correctly, no borderless-table issue. Time-series KPI appendix (pp104-107) has three-year columns, DL-010 time_series_kpi rule superseded by DL-018.</t>
+  </si>
+  <si>
+    <t>Kunlun Energy Company Limited</t>
+  </si>
+  <si>
+    <t>English only (CJK ratio 0.001%, negligible)</t>
+  </si>
+  <si>
+    <t>Two-page-spread layout confirmed again, same DL-012 pattern as ENN (98 PDF pages = up to 190 printed page numbers); severe character-interleaving in extract_text() on pages with vector-drawn diagrams and dense multi-column risk/opportunity tables (BRIGHT ESG model p8, ESG goals petal diagram p13, org-chart diagrams pp30/33/34/36, Net Zero Roadmap p38); extract_tables() on the same pages returns clean cells, so content is recoverable from A1's existing output but A2 does not currently use it; appendix (PDF pg 83-94) cleanly gridlined, no borderless-table issue unlike ENN, DL-015 does not apply; short-term and mid/long-term ESG target tables use the same goal/progress structure as ENN's DL-013 case but that decision is moot under DL-018; very few raster images (56 after size filter) vs earlier firms, consistent with heavy vector-diagram use, which is why this bug was not visible before</t>
+  </si>
+  <si>
+    <t>DL-012 (validated, applies), DL-019 (new)</t>
+  </si>
+  <si>
+    <t>Pages column is PDF count not printed-page-equivalent, same caveat as ENN. Image Objects counted via pdfplumber page.images with a &gt;200x100pt size filter as a proxy for the PyMuPDF method A1 actually uses, so not strictly comparable across firms. Single-char-token ratio (length-1 words / total words) cleanly separates affected pages (39-84%) from document median (2%), used as the detection signal for DL-019. DL-017 referenced in JD Logistics row is missing from both decision log files, flagged, not resolved here.</t>
   </si>
 </sst>
 </file>
@@ -137,12 +152,18 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -360,6 +381,10 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="9" max="9" width="61.5"/>
+    <col customWidth="1" min="11" max="11" width="26.0"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -397,144 +422,254 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>2025.0</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>202.0</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>434431.0</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>971.0</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <v>292.0</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>58.0</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>2025.0</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>150.0</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>436393.0</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>1605.0</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>331.0</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>89.0</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>2025.0</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>79.0</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>897582.0</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>558.0</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="2">
         <v>128.0</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>15.0</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>2025.0</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>115.0</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>965325.0</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>694.0</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="2">
         <v>194.0</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>29.0</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>2025.0</v>
+      </c>
+      <c r="C6" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>406260.0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>2552.0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
+      <c r="Z6" s="3"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>